<commit_message>
Release Pro4.0: refine match-detail columns, invoice numeric preprocess, and full-flush exclude.
Reorder invoice/order detail columns with selective hides; convert invoice qty/price from text; exclude only 已红冲-全额; bump UI to Pro4.0.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/订单数据模板.xlsx
+++ b/templates/订单数据模板.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,16 @@
           <t>用户价格</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>战略标记</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>统计对象</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -493,6 +503,16 @@
       <c r="D2" s="2" t="n">
         <v>113</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>战略</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -511,6 +531,12 @@
       <c r="D3" s="2" t="n">
         <v>226</v>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -528,6 +554,12 @@
       </c>
       <c r="D4" s="2" t="n">
         <v>56.5</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>